<commit_message>
Optimize backend performance, stabilize matching logic, and enhance system logging UI
</commit_message>
<xml_diff>
--- a/test_more.xlsx
+++ b/test_more.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="139">
   <si>
     <t>순번</t>
   </si>
@@ -807,7 +807,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E110"/>
+  <dimension ref="A1:E328"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="3" width="56.625" customWidth="1"/>
@@ -2029,6 +2029,2404 @@
         <v>137</v>
       </c>
     </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A111">
+        <v>110</v>
+      </c>
+      <c r="B111" t="s">
+        <v>5</v>
+      </c>
+      <c r="C111" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A112">
+        <v>111</v>
+      </c>
+      <c r="B112" t="s">
+        <v>7</v>
+      </c>
+      <c r="C112" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A113">
+        <v>112</v>
+      </c>
+      <c r="B113" t="s">
+        <v>9</v>
+      </c>
+      <c r="C113" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A114">
+        <v>113</v>
+      </c>
+      <c r="B114" t="s">
+        <v>11</v>
+      </c>
+      <c r="C114" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A115">
+        <v>114</v>
+      </c>
+      <c r="B115" t="s">
+        <v>13</v>
+      </c>
+      <c r="C115" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A116">
+        <v>115</v>
+      </c>
+      <c r="B116" t="s">
+        <v>15</v>
+      </c>
+      <c r="C116" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A117">
+        <v>116</v>
+      </c>
+      <c r="B117" t="s">
+        <v>17</v>
+      </c>
+      <c r="C117" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A118">
+        <v>117</v>
+      </c>
+      <c r="B118" t="s">
+        <v>19</v>
+      </c>
+      <c r="C118" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A119">
+        <v>118</v>
+      </c>
+      <c r="B119" t="s">
+        <v>21</v>
+      </c>
+      <c r="C119" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A120">
+        <v>119</v>
+      </c>
+      <c r="B120" t="s">
+        <v>23</v>
+      </c>
+      <c r="C120" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A121">
+        <v>120</v>
+      </c>
+      <c r="B121" t="s">
+        <v>25</v>
+      </c>
+      <c r="C121" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A122">
+        <v>121</v>
+      </c>
+      <c r="B122" t="s">
+        <v>27</v>
+      </c>
+      <c r="C122" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A123">
+        <v>122</v>
+      </c>
+      <c r="B123" t="s">
+        <v>29</v>
+      </c>
+      <c r="C123" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A124">
+        <v>123</v>
+      </c>
+      <c r="B124" t="s">
+        <v>138</v>
+      </c>
+      <c r="C124" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A125">
+        <v>124</v>
+      </c>
+      <c r="B125" t="s">
+        <v>32</v>
+      </c>
+      <c r="C125" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A126">
+        <v>125</v>
+      </c>
+      <c r="B126" t="s">
+        <v>27</v>
+      </c>
+      <c r="C126" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A127">
+        <v>126</v>
+      </c>
+      <c r="B127" t="s">
+        <v>29</v>
+      </c>
+      <c r="C127" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A128">
+        <v>127</v>
+      </c>
+      <c r="B128" t="s">
+        <v>36</v>
+      </c>
+      <c r="C128" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A129">
+        <v>128</v>
+      </c>
+      <c r="B129" t="s">
+        <v>27</v>
+      </c>
+      <c r="C129" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A130">
+        <v>129</v>
+      </c>
+      <c r="B130" t="s">
+        <v>39</v>
+      </c>
+      <c r="C130" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A131">
+        <v>130</v>
+      </c>
+      <c r="B131" t="s">
+        <v>41</v>
+      </c>
+      <c r="C131" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A132">
+        <v>131</v>
+      </c>
+      <c r="B132" t="s">
+        <v>43</v>
+      </c>
+      <c r="C132" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A133">
+        <v>132</v>
+      </c>
+      <c r="B133" t="s">
+        <v>36</v>
+      </c>
+      <c r="C133" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A134">
+        <v>133</v>
+      </c>
+      <c r="B134" t="s">
+        <v>46</v>
+      </c>
+      <c r="C134" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A135">
+        <v>134</v>
+      </c>
+      <c r="B135" t="s">
+        <v>36</v>
+      </c>
+      <c r="C135" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A136">
+        <v>135</v>
+      </c>
+      <c r="B136" t="s">
+        <v>49</v>
+      </c>
+      <c r="C136" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A137">
+        <v>136</v>
+      </c>
+      <c r="B137" t="s">
+        <v>51</v>
+      </c>
+      <c r="C137" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A138">
+        <v>137</v>
+      </c>
+      <c r="B138" t="s">
+        <v>138</v>
+      </c>
+      <c r="C138" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A139">
+        <v>138</v>
+      </c>
+      <c r="B139" t="s">
+        <v>25</v>
+      </c>
+      <c r="C139" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A140">
+        <v>139</v>
+      </c>
+      <c r="B140" t="s">
+        <v>27</v>
+      </c>
+      <c r="C140" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A141">
+        <v>140</v>
+      </c>
+      <c r="B141" t="s">
+        <v>29</v>
+      </c>
+      <c r="C141" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A142">
+        <v>141</v>
+      </c>
+      <c r="B142" t="s">
+        <v>51</v>
+      </c>
+      <c r="C142" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A143">
+        <v>142</v>
+      </c>
+      <c r="B143" t="s">
+        <v>25</v>
+      </c>
+      <c r="C143" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A144">
+        <v>143</v>
+      </c>
+      <c r="B144" t="s">
+        <v>49</v>
+      </c>
+      <c r="C144" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A145">
+        <v>144</v>
+      </c>
+      <c r="B145" t="s">
+        <v>43</v>
+      </c>
+      <c r="C145" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A146">
+        <v>145</v>
+      </c>
+      <c r="B146" t="s">
+        <v>61</v>
+      </c>
+      <c r="C146" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A147">
+        <v>146</v>
+      </c>
+      <c r="B147" t="s">
+        <v>32</v>
+      </c>
+      <c r="C147" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A148">
+        <v>147</v>
+      </c>
+      <c r="B148" t="s">
+        <v>46</v>
+      </c>
+      <c r="C148" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A149">
+        <v>148</v>
+      </c>
+      <c r="B149" t="s">
+        <v>27</v>
+      </c>
+      <c r="C149" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A150">
+        <v>149</v>
+      </c>
+      <c r="B150" t="s">
+        <v>66</v>
+      </c>
+      <c r="C150" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A151">
+        <v>150</v>
+      </c>
+      <c r="B151" t="s">
+        <v>39</v>
+      </c>
+      <c r="C151" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A152">
+        <v>151</v>
+      </c>
+      <c r="B152" t="s">
+        <v>66</v>
+      </c>
+      <c r="C152" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A153">
+        <v>152</v>
+      </c>
+      <c r="B153" t="s">
+        <v>41</v>
+      </c>
+      <c r="C153" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A154">
+        <v>153</v>
+      </c>
+      <c r="B154" t="s">
+        <v>36</v>
+      </c>
+      <c r="C154" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A155">
+        <v>154</v>
+      </c>
+      <c r="B155" t="s">
+        <v>36</v>
+      </c>
+      <c r="C155" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A156">
+        <v>155</v>
+      </c>
+      <c r="B156" t="s">
+        <v>23</v>
+      </c>
+      <c r="C156" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A157">
+        <v>156</v>
+      </c>
+      <c r="B157" t="s">
+        <v>27</v>
+      </c>
+      <c r="C157" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A158">
+        <v>157</v>
+      </c>
+      <c r="B158" t="s">
+        <v>51</v>
+      </c>
+      <c r="C158" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A159">
+        <v>158</v>
+      </c>
+      <c r="B159" t="s">
+        <v>61</v>
+      </c>
+      <c r="C159" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A160">
+        <v>159</v>
+      </c>
+      <c r="B160" t="s">
+        <v>46</v>
+      </c>
+      <c r="C160" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A161">
+        <v>160</v>
+      </c>
+      <c r="B161" t="s">
+        <v>29</v>
+      </c>
+      <c r="C161" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A162">
+        <v>161</v>
+      </c>
+      <c r="B162" t="s">
+        <v>78</v>
+      </c>
+      <c r="C162" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A163">
+        <v>162</v>
+      </c>
+      <c r="B163" t="s">
+        <v>78</v>
+      </c>
+      <c r="C163" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A164">
+        <v>163</v>
+      </c>
+      <c r="B164" t="s">
+        <v>46</v>
+      </c>
+      <c r="C164" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A165">
+        <v>164</v>
+      </c>
+      <c r="B165" t="s">
+        <v>81</v>
+      </c>
+      <c r="C165" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A166">
+        <v>165</v>
+      </c>
+      <c r="B166" t="s">
+        <v>43</v>
+      </c>
+      <c r="C166" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A167">
+        <v>166</v>
+      </c>
+      <c r="B167" t="s">
+        <v>84</v>
+      </c>
+      <c r="C167" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A168">
+        <v>167</v>
+      </c>
+      <c r="B168" t="s">
+        <v>23</v>
+      </c>
+      <c r="C168" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A169">
+        <v>168</v>
+      </c>
+      <c r="B169" t="s">
+        <v>138</v>
+      </c>
+      <c r="C169" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A170">
+        <v>169</v>
+      </c>
+      <c r="B170" t="s">
+        <v>66</v>
+      </c>
+      <c r="C170" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A171">
+        <v>170</v>
+      </c>
+      <c r="B171" t="s">
+        <v>23</v>
+      </c>
+      <c r="C171" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A172">
+        <v>171</v>
+      </c>
+      <c r="B172" t="s">
+        <v>89</v>
+      </c>
+      <c r="C172" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A173">
+        <v>172</v>
+      </c>
+      <c r="B173" t="s">
+        <v>32</v>
+      </c>
+      <c r="C173" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A174">
+        <v>173</v>
+      </c>
+      <c r="B174" t="s">
+        <v>36</v>
+      </c>
+      <c r="C174" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A175">
+        <v>174</v>
+      </c>
+      <c r="B175" t="s">
+        <v>93</v>
+      </c>
+      <c r="C175" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A176">
+        <v>175</v>
+      </c>
+      <c r="B176" t="s">
+        <v>29</v>
+      </c>
+      <c r="C176" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A177">
+        <v>176</v>
+      </c>
+      <c r="B177" t="s">
+        <v>89</v>
+      </c>
+      <c r="C177" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A178">
+        <v>177</v>
+      </c>
+      <c r="B178" t="s">
+        <v>43</v>
+      </c>
+      <c r="C178" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A179">
+        <v>178</v>
+      </c>
+      <c r="B179" t="s">
+        <v>78</v>
+      </c>
+      <c r="C179" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A180">
+        <v>179</v>
+      </c>
+      <c r="B180" t="s">
+        <v>43</v>
+      </c>
+      <c r="C180" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A181">
+        <v>180</v>
+      </c>
+      <c r="B181" t="s">
+        <v>49</v>
+      </c>
+      <c r="C181" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A182">
+        <v>181</v>
+      </c>
+      <c r="B182" t="s">
+        <v>36</v>
+      </c>
+      <c r="C182" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A183">
+        <v>182</v>
+      </c>
+      <c r="B183" t="s">
+        <v>138</v>
+      </c>
+      <c r="C183" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A184">
+        <v>183</v>
+      </c>
+      <c r="B184" t="s">
+        <v>25</v>
+      </c>
+      <c r="C184" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A185">
+        <v>184</v>
+      </c>
+      <c r="B185" t="s">
+        <v>51</v>
+      </c>
+      <c r="C185" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A186">
+        <v>185</v>
+      </c>
+      <c r="B186" t="s">
+        <v>61</v>
+      </c>
+      <c r="C186" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A187">
+        <v>186</v>
+      </c>
+      <c r="B187" t="s">
+        <v>66</v>
+      </c>
+      <c r="C187" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A188">
+        <v>187</v>
+      </c>
+      <c r="B188" t="s">
+        <v>27</v>
+      </c>
+      <c r="C188" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A189">
+        <v>188</v>
+      </c>
+      <c r="B189" t="s">
+        <v>61</v>
+      </c>
+      <c r="C189" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A190">
+        <v>189</v>
+      </c>
+      <c r="B190" t="s">
+        <v>41</v>
+      </c>
+      <c r="C190" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A191">
+        <v>190</v>
+      </c>
+      <c r="B191" t="s">
+        <v>49</v>
+      </c>
+      <c r="C191" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A192">
+        <v>191</v>
+      </c>
+      <c r="B192" t="s">
+        <v>39</v>
+      </c>
+      <c r="C192" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A193">
+        <v>192</v>
+      </c>
+      <c r="B193" t="s">
+        <v>49</v>
+      </c>
+      <c r="C193" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A194">
+        <v>193</v>
+      </c>
+      <c r="B194" t="s">
+        <v>36</v>
+      </c>
+      <c r="C194" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A195">
+        <v>194</v>
+      </c>
+      <c r="B195" t="s">
+        <v>41</v>
+      </c>
+      <c r="C195" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A196">
+        <v>195</v>
+      </c>
+      <c r="B196" t="s">
+        <v>23</v>
+      </c>
+      <c r="C196" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A197">
+        <v>196</v>
+      </c>
+      <c r="B197" t="s">
+        <v>49</v>
+      </c>
+      <c r="C197" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A198">
+        <v>197</v>
+      </c>
+      <c r="B198" t="s">
+        <v>36</v>
+      </c>
+      <c r="C198" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A199">
+        <v>198</v>
+      </c>
+      <c r="B199" t="s">
+        <v>29</v>
+      </c>
+      <c r="C199" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A200">
+        <v>199</v>
+      </c>
+      <c r="B200" t="s">
+        <v>93</v>
+      </c>
+      <c r="C200" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A201">
+        <v>200</v>
+      </c>
+      <c r="B201" t="s">
+        <v>43</v>
+      </c>
+      <c r="C201" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A202">
+        <v>201</v>
+      </c>
+      <c r="B202" t="s">
+        <v>23</v>
+      </c>
+      <c r="C202" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A203">
+        <v>202</v>
+      </c>
+      <c r="B203" t="s">
+        <v>61</v>
+      </c>
+      <c r="C203" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A204">
+        <v>203</v>
+      </c>
+      <c r="B204" t="s">
+        <v>81</v>
+      </c>
+      <c r="C204" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A205">
+        <v>204</v>
+      </c>
+      <c r="B205" t="s">
+        <v>66</v>
+      </c>
+      <c r="C205" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A206">
+        <v>205</v>
+      </c>
+      <c r="B206" t="s">
+        <v>29</v>
+      </c>
+      <c r="C206" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A207">
+        <v>206</v>
+      </c>
+      <c r="B207" t="s">
+        <v>66</v>
+      </c>
+      <c r="C207" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A208">
+        <v>207</v>
+      </c>
+      <c r="B208" t="s">
+        <v>23</v>
+      </c>
+      <c r="C208" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A209">
+        <v>208</v>
+      </c>
+      <c r="B209" t="s">
+        <v>29</v>
+      </c>
+      <c r="C209" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A210">
+        <v>209</v>
+      </c>
+      <c r="B210" t="s">
+        <v>51</v>
+      </c>
+      <c r="C210" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A211">
+        <v>210</v>
+      </c>
+      <c r="B211" t="s">
+        <v>49</v>
+      </c>
+      <c r="C211" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A212">
+        <v>211</v>
+      </c>
+      <c r="B212" t="s">
+        <v>46</v>
+      </c>
+      <c r="C212" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A213">
+        <v>212</v>
+      </c>
+      <c r="B213" t="s">
+        <v>93</v>
+      </c>
+      <c r="C213" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A214">
+        <v>213</v>
+      </c>
+      <c r="B214" t="s">
+        <v>23</v>
+      </c>
+      <c r="C214" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A215">
+        <v>214</v>
+      </c>
+      <c r="B215" t="s">
+        <v>36</v>
+      </c>
+      <c r="C215" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A216">
+        <v>215</v>
+      </c>
+      <c r="B216" t="s">
+        <v>89</v>
+      </c>
+      <c r="C216" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A217">
+        <v>216</v>
+      </c>
+      <c r="B217" t="s">
+        <v>49</v>
+      </c>
+      <c r="C217" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A218">
+        <v>217</v>
+      </c>
+      <c r="B218" t="s">
+        <v>29</v>
+      </c>
+      <c r="C218" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A219">
+        <v>218</v>
+      </c>
+      <c r="B219" t="s">
+        <v>81</v>
+      </c>
+      <c r="C219" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A220">
+        <v>219</v>
+      </c>
+      <c r="B220" t="s">
+        <v>5</v>
+      </c>
+      <c r="C220" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A221">
+        <v>220</v>
+      </c>
+      <c r="B221" t="s">
+        <v>7</v>
+      </c>
+      <c r="C221" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A222">
+        <v>221</v>
+      </c>
+      <c r="B222" t="s">
+        <v>9</v>
+      </c>
+      <c r="C222" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A223">
+        <v>222</v>
+      </c>
+      <c r="B223" t="s">
+        <v>11</v>
+      </c>
+      <c r="C223" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A224">
+        <v>223</v>
+      </c>
+      <c r="B224" t="s">
+        <v>13</v>
+      </c>
+      <c r="C224" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A225">
+        <v>224</v>
+      </c>
+      <c r="B225" t="s">
+        <v>15</v>
+      </c>
+      <c r="C225" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A226">
+        <v>225</v>
+      </c>
+      <c r="B226" t="s">
+        <v>17</v>
+      </c>
+      <c r="C226" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A227">
+        <v>226</v>
+      </c>
+      <c r="B227" t="s">
+        <v>19</v>
+      </c>
+      <c r="C227" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A228">
+        <v>227</v>
+      </c>
+      <c r="B228" t="s">
+        <v>21</v>
+      </c>
+      <c r="C228" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A229">
+        <v>228</v>
+      </c>
+      <c r="B229" t="s">
+        <v>23</v>
+      </c>
+      <c r="C229" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A230">
+        <v>229</v>
+      </c>
+      <c r="B230" t="s">
+        <v>25</v>
+      </c>
+      <c r="C230" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A231">
+        <v>230</v>
+      </c>
+      <c r="B231" t="s">
+        <v>27</v>
+      </c>
+      <c r="C231" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A232">
+        <v>231</v>
+      </c>
+      <c r="B232" t="s">
+        <v>29</v>
+      </c>
+      <c r="C232" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A233">
+        <v>232</v>
+      </c>
+      <c r="B233" t="s">
+        <v>138</v>
+      </c>
+      <c r="C233" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A234">
+        <v>233</v>
+      </c>
+      <c r="B234" t="s">
+        <v>32</v>
+      </c>
+      <c r="C234" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A235">
+        <v>234</v>
+      </c>
+      <c r="B235" t="s">
+        <v>27</v>
+      </c>
+      <c r="C235" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A236">
+        <v>235</v>
+      </c>
+      <c r="B236" t="s">
+        <v>29</v>
+      </c>
+      <c r="C236" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A237">
+        <v>236</v>
+      </c>
+      <c r="B237" t="s">
+        <v>36</v>
+      </c>
+      <c r="C237" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A238">
+        <v>237</v>
+      </c>
+      <c r="B238" t="s">
+        <v>27</v>
+      </c>
+      <c r="C238" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="239" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A239">
+        <v>238</v>
+      </c>
+      <c r="B239" t="s">
+        <v>39</v>
+      </c>
+      <c r="C239" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A240">
+        <v>239</v>
+      </c>
+      <c r="B240" t="s">
+        <v>41</v>
+      </c>
+      <c r="C240" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A241">
+        <v>240</v>
+      </c>
+      <c r="B241" t="s">
+        <v>43</v>
+      </c>
+      <c r="C241" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A242">
+        <v>241</v>
+      </c>
+      <c r="B242" t="s">
+        <v>36</v>
+      </c>
+      <c r="C242" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A243">
+        <v>242</v>
+      </c>
+      <c r="B243" t="s">
+        <v>46</v>
+      </c>
+      <c r="C243" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A244">
+        <v>243</v>
+      </c>
+      <c r="B244" t="s">
+        <v>36</v>
+      </c>
+      <c r="C244" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A245">
+        <v>244</v>
+      </c>
+      <c r="B245" t="s">
+        <v>49</v>
+      </c>
+      <c r="C245" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A246">
+        <v>245</v>
+      </c>
+      <c r="B246" t="s">
+        <v>51</v>
+      </c>
+      <c r="C246" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A247">
+        <v>246</v>
+      </c>
+      <c r="B247" t="s">
+        <v>138</v>
+      </c>
+      <c r="C247" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="248" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A248">
+        <v>247</v>
+      </c>
+      <c r="B248" t="s">
+        <v>25</v>
+      </c>
+      <c r="C248" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A249">
+        <v>248</v>
+      </c>
+      <c r="B249" t="s">
+        <v>27</v>
+      </c>
+      <c r="C249" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="250" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A250">
+        <v>249</v>
+      </c>
+      <c r="B250" t="s">
+        <v>29</v>
+      </c>
+      <c r="C250" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="251" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A251">
+        <v>250</v>
+      </c>
+      <c r="B251" t="s">
+        <v>51</v>
+      </c>
+      <c r="C251" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="252" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A252">
+        <v>251</v>
+      </c>
+      <c r="B252" t="s">
+        <v>25</v>
+      </c>
+      <c r="C252" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="253" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A253">
+        <v>252</v>
+      </c>
+      <c r="B253" t="s">
+        <v>49</v>
+      </c>
+      <c r="C253" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="254" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A254">
+        <v>253</v>
+      </c>
+      <c r="B254" t="s">
+        <v>43</v>
+      </c>
+      <c r="C254" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="255" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A255">
+        <v>254</v>
+      </c>
+      <c r="B255" t="s">
+        <v>61</v>
+      </c>
+      <c r="C255" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="256" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A256">
+        <v>255</v>
+      </c>
+      <c r="B256" t="s">
+        <v>32</v>
+      </c>
+      <c r="C256" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A257">
+        <v>256</v>
+      </c>
+      <c r="B257" t="s">
+        <v>46</v>
+      </c>
+      <c r="C257" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A258">
+        <v>257</v>
+      </c>
+      <c r="B258" t="s">
+        <v>27</v>
+      </c>
+      <c r="C258" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A259">
+        <v>258</v>
+      </c>
+      <c r="B259" t="s">
+        <v>66</v>
+      </c>
+      <c r="C259" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A260">
+        <v>259</v>
+      </c>
+      <c r="B260" t="s">
+        <v>39</v>
+      </c>
+      <c r="C260" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="261" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A261">
+        <v>260</v>
+      </c>
+      <c r="B261" t="s">
+        <v>66</v>
+      </c>
+      <c r="C261" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A262">
+        <v>261</v>
+      </c>
+      <c r="B262" t="s">
+        <v>41</v>
+      </c>
+      <c r="C262" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A263">
+        <v>262</v>
+      </c>
+      <c r="B263" t="s">
+        <v>36</v>
+      </c>
+      <c r="C263" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="264" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A264">
+        <v>263</v>
+      </c>
+      <c r="B264" t="s">
+        <v>36</v>
+      </c>
+      <c r="C264" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A265">
+        <v>264</v>
+      </c>
+      <c r="B265" t="s">
+        <v>23</v>
+      </c>
+      <c r="C265" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A266">
+        <v>265</v>
+      </c>
+      <c r="B266" t="s">
+        <v>27</v>
+      </c>
+      <c r="C266" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A267">
+        <v>266</v>
+      </c>
+      <c r="B267" t="s">
+        <v>51</v>
+      </c>
+      <c r="C267" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="268" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A268">
+        <v>267</v>
+      </c>
+      <c r="B268" t="s">
+        <v>61</v>
+      </c>
+      <c r="C268" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A269">
+        <v>268</v>
+      </c>
+      <c r="B269" t="s">
+        <v>46</v>
+      </c>
+      <c r="C269" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="270" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A270">
+        <v>269</v>
+      </c>
+      <c r="B270" t="s">
+        <v>29</v>
+      </c>
+      <c r="C270" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A271">
+        <v>270</v>
+      </c>
+      <c r="B271" t="s">
+        <v>78</v>
+      </c>
+      <c r="C271" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="272" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A272">
+        <v>271</v>
+      </c>
+      <c r="B272" t="s">
+        <v>78</v>
+      </c>
+      <c r="C272" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A273">
+        <v>272</v>
+      </c>
+      <c r="B273" t="s">
+        <v>46</v>
+      </c>
+      <c r="C273" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="274" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A274">
+        <v>273</v>
+      </c>
+      <c r="B274" t="s">
+        <v>81</v>
+      </c>
+      <c r="C274" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="275" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A275">
+        <v>274</v>
+      </c>
+      <c r="B275" t="s">
+        <v>43</v>
+      </c>
+      <c r="C275" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A276">
+        <v>275</v>
+      </c>
+      <c r="B276" t="s">
+        <v>84</v>
+      </c>
+      <c r="C276" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="277" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A277">
+        <v>276</v>
+      </c>
+      <c r="B277" t="s">
+        <v>23</v>
+      </c>
+      <c r="C277" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A278">
+        <v>277</v>
+      </c>
+      <c r="B278" t="s">
+        <v>138</v>
+      </c>
+      <c r="C278" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="279" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A279">
+        <v>278</v>
+      </c>
+      <c r="B279" t="s">
+        <v>66</v>
+      </c>
+      <c r="C279" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="280" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A280">
+        <v>279</v>
+      </c>
+      <c r="B280" t="s">
+        <v>23</v>
+      </c>
+      <c r="C280" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A281">
+        <v>280</v>
+      </c>
+      <c r="B281" t="s">
+        <v>89</v>
+      </c>
+      <c r="C281" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A282">
+        <v>281</v>
+      </c>
+      <c r="B282" t="s">
+        <v>32</v>
+      </c>
+      <c r="C282" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="283" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A283">
+        <v>282</v>
+      </c>
+      <c r="B283" t="s">
+        <v>36</v>
+      </c>
+      <c r="C283" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="284" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A284">
+        <v>283</v>
+      </c>
+      <c r="B284" t="s">
+        <v>93</v>
+      </c>
+      <c r="C284" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="285" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A285">
+        <v>284</v>
+      </c>
+      <c r="B285" t="s">
+        <v>29</v>
+      </c>
+      <c r="C285" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A286">
+        <v>285</v>
+      </c>
+      <c r="B286" t="s">
+        <v>89</v>
+      </c>
+      <c r="C286" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A287">
+        <v>286</v>
+      </c>
+      <c r="B287" t="s">
+        <v>43</v>
+      </c>
+      <c r="C287" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A288">
+        <v>287</v>
+      </c>
+      <c r="B288" t="s">
+        <v>78</v>
+      </c>
+      <c r="C288" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="289" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A289">
+        <v>288</v>
+      </c>
+      <c r="B289" t="s">
+        <v>43</v>
+      </c>
+      <c r="C289" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="290" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A290">
+        <v>289</v>
+      </c>
+      <c r="B290" t="s">
+        <v>49</v>
+      </c>
+      <c r="C290" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="291" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A291">
+        <v>290</v>
+      </c>
+      <c r="B291" t="s">
+        <v>36</v>
+      </c>
+      <c r="C291" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="292" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A292">
+        <v>291</v>
+      </c>
+      <c r="B292" t="s">
+        <v>138</v>
+      </c>
+      <c r="C292" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="293" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A293">
+        <v>292</v>
+      </c>
+      <c r="B293" t="s">
+        <v>25</v>
+      </c>
+      <c r="C293" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="294" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A294">
+        <v>293</v>
+      </c>
+      <c r="B294" t="s">
+        <v>51</v>
+      </c>
+      <c r="C294" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="295" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A295">
+        <v>294</v>
+      </c>
+      <c r="B295" t="s">
+        <v>61</v>
+      </c>
+      <c r="C295" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="296" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A296">
+        <v>295</v>
+      </c>
+      <c r="B296" t="s">
+        <v>66</v>
+      </c>
+      <c r="C296" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A297">
+        <v>296</v>
+      </c>
+      <c r="B297" t="s">
+        <v>27</v>
+      </c>
+      <c r="C297" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A298">
+        <v>297</v>
+      </c>
+      <c r="B298" t="s">
+        <v>61</v>
+      </c>
+      <c r="C298" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A299">
+        <v>298</v>
+      </c>
+      <c r="B299" t="s">
+        <v>41</v>
+      </c>
+      <c r="C299" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A300">
+        <v>299</v>
+      </c>
+      <c r="B300" t="s">
+        <v>49</v>
+      </c>
+      <c r="C300" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A301">
+        <v>300</v>
+      </c>
+      <c r="B301" t="s">
+        <v>39</v>
+      </c>
+      <c r="C301" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A302">
+        <v>301</v>
+      </c>
+      <c r="B302" t="s">
+        <v>49</v>
+      </c>
+      <c r="C302" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A303">
+        <v>302</v>
+      </c>
+      <c r="B303" t="s">
+        <v>36</v>
+      </c>
+      <c r="C303" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A304">
+        <v>303</v>
+      </c>
+      <c r="B304" t="s">
+        <v>41</v>
+      </c>
+      <c r="C304" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A305">
+        <v>304</v>
+      </c>
+      <c r="B305" t="s">
+        <v>23</v>
+      </c>
+      <c r="C305" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A306">
+        <v>305</v>
+      </c>
+      <c r="B306" t="s">
+        <v>49</v>
+      </c>
+      <c r="C306" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A307">
+        <v>306</v>
+      </c>
+      <c r="B307" t="s">
+        <v>36</v>
+      </c>
+      <c r="C307" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A308">
+        <v>307</v>
+      </c>
+      <c r="B308" t="s">
+        <v>29</v>
+      </c>
+      <c r="C308" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A309">
+        <v>308</v>
+      </c>
+      <c r="B309" t="s">
+        <v>93</v>
+      </c>
+      <c r="C309" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A310">
+        <v>309</v>
+      </c>
+      <c r="B310" t="s">
+        <v>43</v>
+      </c>
+      <c r="C310" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A311">
+        <v>310</v>
+      </c>
+      <c r="B311" t="s">
+        <v>23</v>
+      </c>
+      <c r="C311" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A312">
+        <v>311</v>
+      </c>
+      <c r="B312" t="s">
+        <v>61</v>
+      </c>
+      <c r="C312" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A313">
+        <v>312</v>
+      </c>
+      <c r="B313" t="s">
+        <v>81</v>
+      </c>
+      <c r="C313" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A314">
+        <v>313</v>
+      </c>
+      <c r="B314" t="s">
+        <v>66</v>
+      </c>
+      <c r="C314" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A315">
+        <v>314</v>
+      </c>
+      <c r="B315" t="s">
+        <v>29</v>
+      </c>
+      <c r="C315" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A316">
+        <v>315</v>
+      </c>
+      <c r="B316" t="s">
+        <v>66</v>
+      </c>
+      <c r="C316" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A317">
+        <v>316</v>
+      </c>
+      <c r="B317" t="s">
+        <v>23</v>
+      </c>
+      <c r="C317" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A318">
+        <v>317</v>
+      </c>
+      <c r="B318" t="s">
+        <v>29</v>
+      </c>
+      <c r="C318" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A319">
+        <v>318</v>
+      </c>
+      <c r="B319" t="s">
+        <v>51</v>
+      </c>
+      <c r="C319" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A320">
+        <v>319</v>
+      </c>
+      <c r="B320" t="s">
+        <v>49</v>
+      </c>
+      <c r="C320" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="321" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A321">
+        <v>320</v>
+      </c>
+      <c r="B321" t="s">
+        <v>46</v>
+      </c>
+      <c r="C321" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A322">
+        <v>321</v>
+      </c>
+      <c r="B322" t="s">
+        <v>93</v>
+      </c>
+      <c r="C322" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="323" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A323">
+        <v>322</v>
+      </c>
+      <c r="B323" t="s">
+        <v>23</v>
+      </c>
+      <c r="C323" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="324" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A324">
+        <v>323</v>
+      </c>
+      <c r="B324" t="s">
+        <v>36</v>
+      </c>
+      <c r="C324" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="325" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A325">
+        <v>324</v>
+      </c>
+      <c r="B325" t="s">
+        <v>89</v>
+      </c>
+      <c r="C325" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="326" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A326">
+        <v>325</v>
+      </c>
+      <c r="B326" t="s">
+        <v>49</v>
+      </c>
+      <c r="C326" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="327" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A327">
+        <v>326</v>
+      </c>
+      <c r="B327" t="s">
+        <v>29</v>
+      </c>
+      <c r="C327" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A328">
+        <v>327</v>
+      </c>
+      <c r="B328" t="s">
+        <v>81</v>
+      </c>
+      <c r="C328" t="s">
+        <v>137</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Release v1.0 - Stable Administrative District Matching Engine
</commit_message>
<xml_diff>
--- a/test_more.xlsx
+++ b/test_more.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="149">
   <si>
     <t>순번</t>
   </si>
@@ -436,13 +436,45 @@
   </si>
   <si>
     <t>강원도 홍천군 두촌면 괘석리</t>
+  </si>
+  <si>
+    <t>전북특별자치도 부안군 위도면 상왕등리</t>
+  </si>
+  <si>
+    <t>강원특별자치도 고성군 죽왕면 오봉리</t>
+  </si>
+  <si>
+    <t>울산광역시 울주군 두동면 구미리</t>
+  </si>
+  <si>
+    <t>대구광역시 달성군 하빈면 무등리</t>
+  </si>
+  <si>
+    <t>광주광역시 서구 세하동</t>
+  </si>
+  <si>
+    <t>대전광역시 동구 오동</t>
+  </si>
+  <si>
+    <t>울산광역시 중구 남외동</t>
+  </si>
+  <si>
+    <t>부산광역시 기장군 장안읍 장안리</t>
+  </si>
+  <si>
+    <t>제주특별자치도 제주시 애월읍 상가리</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>제주도 북제주군 구좌면 동복리</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -464,16 +496,28 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF565656"/>
+      <name val="NanumGothic"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -496,14 +540,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color rgb="FF1E74BF"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -807,13 +869,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E328"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E329"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="2" max="3" width="56.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -830,7 +892,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -841,7 +903,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>2</v>
       </c>
@@ -852,7 +914,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>3</v>
       </c>
@@ -863,7 +925,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -874,7 +936,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5">
       <c r="A6">
         <v>5</v>
       </c>
@@ -885,7 +947,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5">
       <c r="A7">
         <v>6</v>
       </c>
@@ -896,7 +958,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5">
       <c r="A8">
         <v>7</v>
       </c>
@@ -907,7 +969,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5">
       <c r="A9">
         <v>8</v>
       </c>
@@ -918,7 +980,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5">
       <c r="A10">
         <v>9</v>
       </c>
@@ -929,7 +991,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5">
       <c r="A11">
         <v>10</v>
       </c>
@@ -940,7 +1002,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5">
       <c r="A12">
         <v>11</v>
       </c>
@@ -951,7 +1013,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5">
       <c r="A13">
         <v>12</v>
       </c>
@@ -962,7 +1024,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5">
       <c r="A14">
         <v>13</v>
       </c>
@@ -973,7 +1035,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5">
       <c r="A15">
         <v>14</v>
       </c>
@@ -984,7 +1046,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5">
       <c r="A16">
         <v>15</v>
       </c>
@@ -995,7 +1057,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1006,117 +1068,117 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>148</v>
       </c>
       <c r="C18" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>36</v>
+        <v>147</v>
       </c>
       <c r="C19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" ht="17.25" thickBot="1">
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
-        <v>27</v>
+      <c r="B20" s="2" t="s">
+        <v>139</v>
       </c>
       <c r="C20" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="18" thickTop="1" thickBot="1">
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
-        <v>39</v>
+      <c r="B21" s="4" t="s">
+        <v>140</v>
       </c>
       <c r="C21" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" t="s">
-        <v>41</v>
+      <c r="B22" s="2" t="s">
+        <v>141</v>
       </c>
       <c r="C22" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" ht="17.25" thickBot="1">
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" t="s">
-        <v>43</v>
+      <c r="B23" s="2" t="s">
+        <v>142</v>
       </c>
       <c r="C23" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="18" thickTop="1" thickBot="1">
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24" t="s">
-        <v>36</v>
+      <c r="B24" s="4" t="s">
+        <v>143</v>
       </c>
       <c r="C24" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3">
       <c r="A25">
         <v>24</v>
       </c>
-      <c r="B25" t="s">
-        <v>46</v>
+      <c r="B25" s="2" t="s">
+        <v>144</v>
       </c>
       <c r="C25" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="17.25" thickBot="1">
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26" t="s">
-        <v>36</v>
+      <c r="B26" s="2" t="s">
+        <v>145</v>
       </c>
       <c r="C26" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" ht="18" thickTop="1" thickBot="1">
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" t="s">
-        <v>49</v>
+      <c r="B27" s="4" t="s">
+        <v>146</v>
       </c>
       <c r="C27" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1127,7 +1189,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1138,7 +1200,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1149,7 +1211,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1160,7 +1222,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1171,7 +1233,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1182,7 +1244,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1193,7 +1255,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1204,7 +1266,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1215,7 +1277,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1226,7 +1288,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1237,7 +1299,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1248,7 +1310,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1259,7 +1321,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1270,7 +1332,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1281,7 +1343,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1292,7 +1354,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1303,7 +1365,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1314,7 +1376,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1325,7 +1387,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1336,7 +1398,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1347,7 +1409,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1358,7 +1420,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1369,7 +1431,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1380,7 +1442,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1391,7 +1453,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1402,7 +1464,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1413,7 +1475,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1424,7 +1486,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1435,7 +1497,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1446,7 +1508,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1457,7 +1519,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -1468,7 +1530,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -1479,7 +1541,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -1490,7 +1552,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3">
       <c r="A62">
         <v>61</v>
       </c>
@@ -1501,7 +1563,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3">
       <c r="A63">
         <v>62</v>
       </c>
@@ -1512,7 +1574,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3">
       <c r="A64">
         <v>63</v>
       </c>
@@ -1523,7 +1585,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3">
       <c r="A65">
         <v>64</v>
       </c>
@@ -1534,7 +1596,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3">
       <c r="A66">
         <v>65</v>
       </c>
@@ -1545,7 +1607,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3">
       <c r="A67">
         <v>66</v>
       </c>
@@ -1556,7 +1618,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3">
       <c r="A68">
         <v>67</v>
       </c>
@@ -1567,7 +1629,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:3">
       <c r="A69">
         <v>68</v>
       </c>
@@ -1578,7 +1640,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3">
       <c r="A70">
         <v>69</v>
       </c>
@@ -1589,7 +1651,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:3">
       <c r="A71">
         <v>70</v>
       </c>
@@ -1600,7 +1662,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:3">
       <c r="A72">
         <v>71</v>
       </c>
@@ -1611,7 +1673,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:3">
       <c r="A73">
         <v>72</v>
       </c>
@@ -1622,7 +1684,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:3">
       <c r="A74">
         <v>73</v>
       </c>
@@ -1633,7 +1695,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:3">
       <c r="A75">
         <v>74</v>
       </c>
@@ -1644,7 +1706,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:3">
       <c r="A76">
         <v>75</v>
       </c>
@@ -1655,7 +1717,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3">
       <c r="A77">
         <v>76</v>
       </c>
@@ -1666,7 +1728,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:3">
       <c r="A78">
         <v>77</v>
       </c>
@@ -1677,7 +1739,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:3">
       <c r="A79">
         <v>78</v>
       </c>
@@ -1688,7 +1750,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:3">
       <c r="A80">
         <v>79</v>
       </c>
@@ -1699,7 +1761,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:3">
       <c r="A81">
         <v>80</v>
       </c>
@@ -1710,7 +1772,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3">
       <c r="A82">
         <v>81</v>
       </c>
@@ -1721,7 +1783,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:3">
       <c r="A83">
         <v>82</v>
       </c>
@@ -1732,7 +1794,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3">
       <c r="A84">
         <v>83</v>
       </c>
@@ -1743,7 +1805,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3">
       <c r="A85">
         <v>84</v>
       </c>
@@ -1754,7 +1816,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3">
       <c r="A86">
         <v>85</v>
       </c>
@@ -1765,7 +1827,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3">
       <c r="A87">
         <v>86</v>
       </c>
@@ -1776,7 +1838,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3">
       <c r="A88">
         <v>87</v>
       </c>
@@ -1787,7 +1849,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3">
       <c r="A89">
         <v>88</v>
       </c>
@@ -1798,7 +1860,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3">
       <c r="A90">
         <v>89</v>
       </c>
@@ -1809,7 +1871,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:3">
       <c r="A91">
         <v>90</v>
       </c>
@@ -1820,7 +1882,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:3">
       <c r="A92">
         <v>91</v>
       </c>
@@ -1831,7 +1893,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3">
       <c r="A93">
         <v>92</v>
       </c>
@@ -1842,7 +1904,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:3">
       <c r="A94">
         <v>93</v>
       </c>
@@ -1853,7 +1915,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3">
       <c r="A95">
         <v>94</v>
       </c>
@@ -1864,7 +1926,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3">
       <c r="A96">
         <v>95</v>
       </c>
@@ -1875,7 +1937,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:3">
       <c r="A97">
         <v>96</v>
       </c>
@@ -1886,7 +1948,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:3">
       <c r="A98">
         <v>97</v>
       </c>
@@ -1897,7 +1959,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:3">
       <c r="A99">
         <v>98</v>
       </c>
@@ -1908,7 +1970,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:3">
       <c r="A100">
         <v>99</v>
       </c>
@@ -1919,7 +1981,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:3">
       <c r="A101">
         <v>100</v>
       </c>
@@ -1930,7 +1992,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:3">
       <c r="A102">
         <v>101</v>
       </c>
@@ -1941,7 +2003,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:3">
       <c r="A103">
         <v>102</v>
       </c>
@@ -1952,7 +2014,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:3">
       <c r="A104">
         <v>103</v>
       </c>
@@ -1963,7 +2025,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:3">
       <c r="A105">
         <v>104</v>
       </c>
@@ -1974,7 +2036,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:3">
       <c r="A106">
         <v>105</v>
       </c>
@@ -1985,7 +2047,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:3">
       <c r="A107">
         <v>106</v>
       </c>
@@ -1996,7 +2058,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:3">
       <c r="A108">
         <v>107</v>
       </c>
@@ -2007,7 +2069,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:3">
       <c r="A109">
         <v>108</v>
       </c>
@@ -2018,7 +2080,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:3">
       <c r="A110">
         <v>109</v>
       </c>
@@ -2029,7 +2091,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:3">
       <c r="A111">
         <v>110</v>
       </c>
@@ -2040,7 +2102,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:3">
       <c r="A112">
         <v>111</v>
       </c>
@@ -2051,7 +2113,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:3">
       <c r="A113">
         <v>112</v>
       </c>
@@ -2062,7 +2124,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:3">
       <c r="A114">
         <v>113</v>
       </c>
@@ -2073,7 +2135,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:3">
       <c r="A115">
         <v>114</v>
       </c>
@@ -2084,7 +2146,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:3">
       <c r="A116">
         <v>115</v>
       </c>
@@ -2095,7 +2157,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:3">
       <c r="A117">
         <v>116</v>
       </c>
@@ -2106,7 +2168,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:3">
       <c r="A118">
         <v>117</v>
       </c>
@@ -2117,7 +2179,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:3">
       <c r="A119">
         <v>118</v>
       </c>
@@ -2128,7 +2190,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:3">
       <c r="A120">
         <v>119</v>
       </c>
@@ -2139,7 +2201,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:3">
       <c r="A121">
         <v>120</v>
       </c>
@@ -2150,7 +2212,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:3">
       <c r="A122">
         <v>121</v>
       </c>
@@ -2161,7 +2223,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:3">
       <c r="A123">
         <v>122</v>
       </c>
@@ -2172,7 +2234,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:3">
       <c r="A124">
         <v>123</v>
       </c>
@@ -2183,7 +2245,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:3">
       <c r="A125">
         <v>124</v>
       </c>
@@ -2194,7 +2256,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:3">
       <c r="A126">
         <v>125</v>
       </c>
@@ -2205,7 +2267,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:3">
       <c r="A127">
         <v>126</v>
       </c>
@@ -2216,7 +2278,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:3">
       <c r="A128">
         <v>127</v>
       </c>
@@ -2227,7 +2289,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:3">
       <c r="A129">
         <v>128</v>
       </c>
@@ -2238,7 +2300,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:3">
       <c r="A130">
         <v>129</v>
       </c>
@@ -2249,7 +2311,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:3">
       <c r="A131">
         <v>130</v>
       </c>
@@ -2260,7 +2322,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:3">
       <c r="A132">
         <v>131</v>
       </c>
@@ -2271,7 +2333,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:3">
       <c r="A133">
         <v>132</v>
       </c>
@@ -2282,7 +2344,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:3">
       <c r="A134">
         <v>133</v>
       </c>
@@ -2293,7 +2355,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:3">
       <c r="A135">
         <v>134</v>
       </c>
@@ -2304,7 +2366,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:3">
       <c r="A136">
         <v>135</v>
       </c>
@@ -2315,7 +2377,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:3">
       <c r="A137">
         <v>136</v>
       </c>
@@ -2326,7 +2388,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:3">
       <c r="A138">
         <v>137</v>
       </c>
@@ -2337,7 +2399,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:3">
       <c r="A139">
         <v>138</v>
       </c>
@@ -2348,7 +2410,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:3">
       <c r="A140">
         <v>139</v>
       </c>
@@ -2359,7 +2421,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:3">
       <c r="A141">
         <v>140</v>
       </c>
@@ -2370,7 +2432,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:3">
       <c r="A142">
         <v>141</v>
       </c>
@@ -2381,7 +2443,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:3">
       <c r="A143">
         <v>142</v>
       </c>
@@ -2392,7 +2454,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:3">
       <c r="A144">
         <v>143</v>
       </c>
@@ -2403,7 +2465,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:3">
       <c r="A145">
         <v>144</v>
       </c>
@@ -2414,7 +2476,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:3">
       <c r="A146">
         <v>145</v>
       </c>
@@ -2425,7 +2487,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:3">
       <c r="A147">
         <v>146</v>
       </c>
@@ -2436,7 +2498,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:3">
       <c r="A148">
         <v>147</v>
       </c>
@@ -2447,7 +2509,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:3">
       <c r="A149">
         <v>148</v>
       </c>
@@ -2458,7 +2520,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:3">
       <c r="A150">
         <v>149</v>
       </c>
@@ -2469,7 +2531,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:3">
       <c r="A151">
         <v>150</v>
       </c>
@@ -2480,7 +2542,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:3">
       <c r="A152">
         <v>151</v>
       </c>
@@ -2491,7 +2553,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:3">
       <c r="A153">
         <v>152</v>
       </c>
@@ -2502,7 +2564,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:3">
       <c r="A154">
         <v>153</v>
       </c>
@@ -2513,7 +2575,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:3">
       <c r="A155">
         <v>154</v>
       </c>
@@ -2524,7 +2586,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:3">
       <c r="A156">
         <v>155</v>
       </c>
@@ -2535,7 +2597,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:3">
       <c r="A157">
         <v>156</v>
       </c>
@@ -2546,7 +2608,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:3">
       <c r="A158">
         <v>157</v>
       </c>
@@ -2557,7 +2619,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:3">
       <c r="A159">
         <v>158</v>
       </c>
@@ -2568,7 +2630,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:3">
       <c r="A160">
         <v>159</v>
       </c>
@@ -2579,7 +2641,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:3">
       <c r="A161">
         <v>160</v>
       </c>
@@ -2590,7 +2652,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:3">
       <c r="A162">
         <v>161</v>
       </c>
@@ -2601,7 +2663,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:3">
       <c r="A163">
         <v>162</v>
       </c>
@@ -2612,7 +2674,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:3">
       <c r="A164">
         <v>163</v>
       </c>
@@ -2623,7 +2685,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:3">
       <c r="A165">
         <v>164</v>
       </c>
@@ -2634,7 +2696,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:3">
       <c r="A166">
         <v>165</v>
       </c>
@@ -2645,7 +2707,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:3">
       <c r="A167">
         <v>166</v>
       </c>
@@ -2656,7 +2718,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:3">
       <c r="A168">
         <v>167</v>
       </c>
@@ -2667,7 +2729,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:3">
       <c r="A169">
         <v>168</v>
       </c>
@@ -2678,7 +2740,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:3">
       <c r="A170">
         <v>169</v>
       </c>
@@ -2689,7 +2751,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:3">
       <c r="A171">
         <v>170</v>
       </c>
@@ -2700,7 +2762,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:3">
       <c r="A172">
         <v>171</v>
       </c>
@@ -2711,7 +2773,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:3">
       <c r="A173">
         <v>172</v>
       </c>
@@ -2722,7 +2784,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:3">
       <c r="A174">
         <v>173</v>
       </c>
@@ -2733,7 +2795,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:3">
       <c r="A175">
         <v>174</v>
       </c>
@@ -2744,7 +2806,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:3">
       <c r="A176">
         <v>175</v>
       </c>
@@ -2755,7 +2817,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:3">
       <c r="A177">
         <v>176</v>
       </c>
@@ -2766,7 +2828,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:3">
       <c r="A178">
         <v>177</v>
       </c>
@@ -2777,7 +2839,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:3">
       <c r="A179">
         <v>178</v>
       </c>
@@ -2788,7 +2850,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:3">
       <c r="A180">
         <v>179</v>
       </c>
@@ -2799,7 +2861,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:3">
       <c r="A181">
         <v>180</v>
       </c>
@@ -2810,7 +2872,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:3">
       <c r="A182">
         <v>181</v>
       </c>
@@ -2821,7 +2883,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:3">
       <c r="A183">
         <v>182</v>
       </c>
@@ -2832,7 +2894,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:3">
       <c r="A184">
         <v>183</v>
       </c>
@@ -2843,7 +2905,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:3">
       <c r="A185">
         <v>184</v>
       </c>
@@ -2854,7 +2916,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:3">
       <c r="A186">
         <v>185</v>
       </c>
@@ -2865,7 +2927,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:3">
       <c r="A187">
         <v>186</v>
       </c>
@@ -2876,7 +2938,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:3">
       <c r="A188">
         <v>187</v>
       </c>
@@ -2887,7 +2949,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:3">
       <c r="A189">
         <v>188</v>
       </c>
@@ -2898,7 +2960,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:3">
       <c r="A190">
         <v>189</v>
       </c>
@@ -2909,7 +2971,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:3">
       <c r="A191">
         <v>190</v>
       </c>
@@ -2920,7 +2982,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:3">
       <c r="A192">
         <v>191</v>
       </c>
@@ -2931,7 +2993,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:3">
       <c r="A193">
         <v>192</v>
       </c>
@@ -2942,7 +3004,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:3">
       <c r="A194">
         <v>193</v>
       </c>
@@ -2953,7 +3015,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:3">
       <c r="A195">
         <v>194</v>
       </c>
@@ -2964,7 +3026,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:3">
       <c r="A196">
         <v>195</v>
       </c>
@@ -2975,7 +3037,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:3">
       <c r="A197">
         <v>196</v>
       </c>
@@ -2986,7 +3048,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:3">
       <c r="A198">
         <v>197</v>
       </c>
@@ -2997,7 +3059,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:3">
       <c r="A199">
         <v>198</v>
       </c>
@@ -3008,7 +3070,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:3">
       <c r="A200">
         <v>199</v>
       </c>
@@ -3019,7 +3081,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:3">
       <c r="A201">
         <v>200</v>
       </c>
@@ -3030,7 +3092,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:3">
       <c r="A202">
         <v>201</v>
       </c>
@@ -3041,7 +3103,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:3">
       <c r="A203">
         <v>202</v>
       </c>
@@ -3052,7 +3114,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:3">
       <c r="A204">
         <v>203</v>
       </c>
@@ -3063,7 +3125,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:3">
       <c r="A205">
         <v>204</v>
       </c>
@@ -3074,7 +3136,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:3">
       <c r="A206">
         <v>205</v>
       </c>
@@ -3085,7 +3147,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:3">
       <c r="A207">
         <v>206</v>
       </c>
@@ -3096,7 +3158,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:3">
       <c r="A208">
         <v>207</v>
       </c>
@@ -3107,7 +3169,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:3">
       <c r="A209">
         <v>208</v>
       </c>
@@ -3118,7 +3180,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:3">
       <c r="A210">
         <v>209</v>
       </c>
@@ -3129,7 +3191,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:3">
       <c r="A211">
         <v>210</v>
       </c>
@@ -3140,7 +3202,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:3">
       <c r="A212">
         <v>211</v>
       </c>
@@ -3151,7 +3213,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:3">
       <c r="A213">
         <v>212</v>
       </c>
@@ -3162,7 +3224,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:3">
       <c r="A214">
         <v>213</v>
       </c>
@@ -3173,7 +3235,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:3">
       <c r="A215">
         <v>214</v>
       </c>
@@ -3184,7 +3246,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:3">
       <c r="A216">
         <v>215</v>
       </c>
@@ -3195,7 +3257,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:3">
       <c r="A217">
         <v>216</v>
       </c>
@@ -3206,7 +3268,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:3">
       <c r="A218">
         <v>217</v>
       </c>
@@ -3217,7 +3279,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:3">
       <c r="A219">
         <v>218</v>
       </c>
@@ -3228,7 +3290,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:3">
       <c r="A220">
         <v>219</v>
       </c>
@@ -3239,7 +3301,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:3">
       <c r="A221">
         <v>220</v>
       </c>
@@ -3250,7 +3312,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:3">
       <c r="A222">
         <v>221</v>
       </c>
@@ -3261,7 +3323,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:3">
       <c r="A223">
         <v>222</v>
       </c>
@@ -3272,7 +3334,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:3">
       <c r="A224">
         <v>223</v>
       </c>
@@ -3283,7 +3345,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:3">
       <c r="A225">
         <v>224</v>
       </c>
@@ -3294,7 +3356,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:3">
       <c r="A226">
         <v>225</v>
       </c>
@@ -3305,7 +3367,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:3">
       <c r="A227">
         <v>226</v>
       </c>
@@ -3316,7 +3378,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:3">
       <c r="A228">
         <v>227</v>
       </c>
@@ -3327,7 +3389,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:3">
       <c r="A229">
         <v>228</v>
       </c>
@@ -3338,7 +3400,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:3">
       <c r="A230">
         <v>229</v>
       </c>
@@ -3349,7 +3411,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:3">
       <c r="A231">
         <v>230</v>
       </c>
@@ -3360,7 +3422,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:3">
       <c r="A232">
         <v>231</v>
       </c>
@@ -3371,7 +3433,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:3">
       <c r="A233">
         <v>232</v>
       </c>
@@ -3382,7 +3444,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:3">
       <c r="A234">
         <v>233</v>
       </c>
@@ -3393,7 +3455,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:3">
       <c r="A235">
         <v>234</v>
       </c>
@@ -3404,7 +3466,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:3">
       <c r="A236">
         <v>235</v>
       </c>
@@ -3415,7 +3477,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:3">
       <c r="A237">
         <v>236</v>
       </c>
@@ -3426,7 +3488,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:3">
       <c r="A238">
         <v>237</v>
       </c>
@@ -3437,7 +3499,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:3">
       <c r="A239">
         <v>238</v>
       </c>
@@ -3448,7 +3510,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:3">
       <c r="A240">
         <v>239</v>
       </c>
@@ -3459,7 +3521,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="241" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:3">
       <c r="A241">
         <v>240</v>
       </c>
@@ -3470,7 +3532,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:3">
       <c r="A242">
         <v>241</v>
       </c>
@@ -3481,7 +3543,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:3">
       <c r="A243">
         <v>242</v>
       </c>
@@ -3492,7 +3554,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:3">
       <c r="A244">
         <v>243</v>
       </c>
@@ -3503,7 +3565,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:3">
       <c r="A245">
         <v>244</v>
       </c>
@@ -3514,7 +3576,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:3">
       <c r="A246">
         <v>245</v>
       </c>
@@ -3525,7 +3587,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:3">
       <c r="A247">
         <v>246</v>
       </c>
@@ -3536,7 +3598,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:3">
       <c r="A248">
         <v>247</v>
       </c>
@@ -3547,7 +3609,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:3">
       <c r="A249">
         <v>248</v>
       </c>
@@ -3558,7 +3620,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:3">
       <c r="A250">
         <v>249</v>
       </c>
@@ -3569,7 +3631,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:3">
       <c r="A251">
         <v>250</v>
       </c>
@@ -3580,7 +3642,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:3">
       <c r="A252">
         <v>251</v>
       </c>
@@ -3591,7 +3653,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="253" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:3">
       <c r="A253">
         <v>252</v>
       </c>
@@ -3602,7 +3664,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:3">
       <c r="A254">
         <v>253</v>
       </c>
@@ -3613,7 +3675,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:3">
       <c r="A255">
         <v>254</v>
       </c>
@@ -3624,7 +3686,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:3">
       <c r="A256">
         <v>255</v>
       </c>
@@ -3635,7 +3697,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:3">
       <c r="A257">
         <v>256</v>
       </c>
@@ -3646,7 +3708,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="258" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:3">
       <c r="A258">
         <v>257</v>
       </c>
@@ -3657,7 +3719,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:3">
       <c r="A259">
         <v>258</v>
       </c>
@@ -3668,7 +3730,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:3">
       <c r="A260">
         <v>259</v>
       </c>
@@ -3679,7 +3741,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:3">
       <c r="A261">
         <v>260</v>
       </c>
@@ -3690,7 +3752,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:3">
       <c r="A262">
         <v>261</v>
       </c>
@@ -3701,7 +3763,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:3">
       <c r="A263">
         <v>262</v>
       </c>
@@ -3712,7 +3774,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="264" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:3">
       <c r="A264">
         <v>263</v>
       </c>
@@ -3723,7 +3785,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:3">
       <c r="A265">
         <v>264</v>
       </c>
@@ -3734,7 +3796,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:3">
       <c r="A266">
         <v>265</v>
       </c>
@@ -3745,7 +3807,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:3">
       <c r="A267">
         <v>266</v>
       </c>
@@ -3756,7 +3818,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:3">
       <c r="A268">
         <v>267</v>
       </c>
@@ -3767,7 +3829,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:3">
       <c r="A269">
         <v>268</v>
       </c>
@@ -3778,7 +3840,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="270" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:3">
       <c r="A270">
         <v>269</v>
       </c>
@@ -3789,7 +3851,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:3">
       <c r="A271">
         <v>270</v>
       </c>
@@ -3800,7 +3862,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="272" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:3">
       <c r="A272">
         <v>271</v>
       </c>
@@ -3811,7 +3873,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:3">
       <c r="A273">
         <v>272</v>
       </c>
@@ -3822,7 +3884,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:3">
       <c r="A274">
         <v>273</v>
       </c>
@@ -3833,7 +3895,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="275" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:3">
       <c r="A275">
         <v>274</v>
       </c>
@@ -3844,7 +3906,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:3">
       <c r="A276">
         <v>275</v>
       </c>
@@ -3855,7 +3917,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="277" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:3">
       <c r="A277">
         <v>276</v>
       </c>
@@ -3866,7 +3928,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:3">
       <c r="A278">
         <v>277</v>
       </c>
@@ -3877,7 +3939,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="279" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:3">
       <c r="A279">
         <v>278</v>
       </c>
@@ -3888,7 +3950,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="280" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:3">
       <c r="A280">
         <v>279</v>
       </c>
@@ -3899,7 +3961,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:3">
       <c r="A281">
         <v>280</v>
       </c>
@@ -3910,7 +3972,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:3">
       <c r="A282">
         <v>281</v>
       </c>
@@ -3921,7 +3983,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="283" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:3">
       <c r="A283">
         <v>282</v>
       </c>
@@ -3932,7 +3994,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="284" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:3">
       <c r="A284">
         <v>283</v>
       </c>
@@ -3943,7 +4005,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="285" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:3">
       <c r="A285">
         <v>284</v>
       </c>
@@ -3954,7 +4016,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="286" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:3">
       <c r="A286">
         <v>285</v>
       </c>
@@ -3965,7 +4027,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="287" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:3">
       <c r="A287">
         <v>286</v>
       </c>
@@ -3976,7 +4038,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="288" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:3">
       <c r="A288">
         <v>287</v>
       </c>
@@ -3987,7 +4049,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="289" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:3">
       <c r="A289">
         <v>288</v>
       </c>
@@ -3998,7 +4060,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:3">
       <c r="A290">
         <v>289</v>
       </c>
@@ -4009,7 +4071,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="291" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:3">
       <c r="A291">
         <v>290</v>
       </c>
@@ -4020,7 +4082,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="292" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:3">
       <c r="A292">
         <v>291</v>
       </c>
@@ -4031,7 +4093,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="293" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:3">
       <c r="A293">
         <v>292</v>
       </c>
@@ -4042,7 +4104,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="294" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:3">
       <c r="A294">
         <v>293</v>
       </c>
@@ -4053,7 +4115,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="295" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:3">
       <c r="A295">
         <v>294</v>
       </c>
@@ -4064,7 +4126,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="296" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:3">
       <c r="A296">
         <v>295</v>
       </c>
@@ -4075,7 +4137,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="297" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:3">
       <c r="A297">
         <v>296</v>
       </c>
@@ -4086,7 +4148,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="298" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:3">
       <c r="A298">
         <v>297</v>
       </c>
@@ -4097,7 +4159,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="299" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:3">
       <c r="A299">
         <v>298</v>
       </c>
@@ -4108,7 +4170,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="300" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:3">
       <c r="A300">
         <v>299</v>
       </c>
@@ -4119,7 +4181,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="301" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:3">
       <c r="A301">
         <v>300</v>
       </c>
@@ -4130,7 +4192,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="302" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:3">
       <c r="A302">
         <v>301</v>
       </c>
@@ -4141,7 +4203,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="303" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:3">
       <c r="A303">
         <v>302</v>
       </c>
@@ -4152,7 +4214,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:3">
       <c r="A304">
         <v>303</v>
       </c>
@@ -4163,7 +4225,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:3">
       <c r="A305">
         <v>304</v>
       </c>
@@ -4174,7 +4236,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="306" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:3">
       <c r="A306">
         <v>305</v>
       </c>
@@ -4185,7 +4247,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="307" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:3">
       <c r="A307">
         <v>306</v>
       </c>
@@ -4196,7 +4258,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="308" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:3">
       <c r="A308">
         <v>307</v>
       </c>
@@ -4207,7 +4269,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="309" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:3">
       <c r="A309">
         <v>308</v>
       </c>
@@ -4218,7 +4280,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="310" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:3">
       <c r="A310">
         <v>309</v>
       </c>
@@ -4229,7 +4291,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="311" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:3">
       <c r="A311">
         <v>310</v>
       </c>
@@ -4240,7 +4302,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="312" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:3">
       <c r="A312">
         <v>311</v>
       </c>
@@ -4251,7 +4313,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:3">
       <c r="A313">
         <v>312</v>
       </c>
@@ -4262,7 +4324,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:3">
       <c r="A314">
         <v>313</v>
       </c>
@@ -4273,7 +4335,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="315" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:3">
       <c r="A315">
         <v>314</v>
       </c>
@@ -4284,7 +4346,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="316" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:3">
       <c r="A316">
         <v>315</v>
       </c>
@@ -4295,7 +4357,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="317" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:3">
       <c r="A317">
         <v>316</v>
       </c>
@@ -4306,7 +4368,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="318" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:3">
       <c r="A318">
         <v>317</v>
       </c>
@@ -4317,7 +4379,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="319" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:3">
       <c r="A319">
         <v>318</v>
       </c>
@@ -4328,7 +4390,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="320" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:3">
       <c r="A320">
         <v>319</v>
       </c>
@@ -4339,7 +4401,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="321" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:3">
       <c r="A321">
         <v>320</v>
       </c>
@@ -4350,7 +4412,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="322" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:3">
       <c r="A322">
         <v>321</v>
       </c>
@@ -4361,7 +4423,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="323" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:3">
       <c r="A323">
         <v>322</v>
       </c>
@@ -4372,7 +4434,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="324" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:3">
       <c r="A324">
         <v>323</v>
       </c>
@@ -4383,7 +4445,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="325" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:3">
       <c r="A325">
         <v>324</v>
       </c>
@@ -4394,7 +4456,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="326" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:3">
       <c r="A326">
         <v>325</v>
       </c>
@@ -4405,7 +4467,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="327" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:3">
       <c r="A327">
         <v>326</v>
       </c>
@@ -4416,7 +4478,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="328" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:3">
       <c r="A328">
         <v>327</v>
       </c>
@@ -4426,6 +4488,9 @@
       <c r="C328" t="s">
         <v>137</v>
       </c>
+    </row>
+    <row r="329" spans="1:3">
+      <c r="C329" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>